<commit_message>
Fix gross margin denominator: use operating revenue (not total)
การเทียบ DUSIT MD&A เผยว่า GM ควรหารด้วยรายได้ดำเนินงาน ไม่ใช่รายได้รวม:
- เดิม: (รายได้รวม−ต้นทุน)/รายได้รวม = 39.7% (รวมรายได้อื่นในตัวหาร)
- แก้: (รายได้ดำเนินงาน−ต้นทุน)/รายได้ดำเนินงาน = 32.0% ตรง DUSIT 31.5%
NPM/ROA/ROE คงใช้รายได้รวม (มาตรฐาน ตรงบริษัทอยู่แล้ว)

DSO ที่ต่าง = นิยาม (เราใช้ลูกหนี้การค้า+อื่นตามหน้างบ; บริษัทใช้ลูกหนี้การค้า
ล้วนจากหมายเหตุ) ไม่ใช่บั๊ก - ใช้นิยามเดียวสม่ำเสมอทุกบริษัท

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WjBjdz26s52MeASaozo8gq
</commit_message>
<xml_diff>
--- a/tour-finance/output/ratios_report.xlsx
+++ b/tour-finance/output/ratios_report.xlsx
@@ -525,7 +525,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>30.9%</t>
+          <t>26.6%</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -569,7 +569,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>46.7%</t>
+          <t>44.2%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -613,7 +613,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>39.7%</t>
+          <t>32.0%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -657,7 +657,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>58.9%</t>
+          <t>58.7%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>41.2%</t>
+          <t>41.0%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -745,7 +745,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>48.0%</t>
+          <t>46.6%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -833,7 +833,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>67.7%</t>
+          <t>67.4%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -877,7 +877,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>39.7%</t>
+          <t>39.0%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>45.1%</t>
+          <t>43.4%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">

</xml_diff>

<commit_message>
Add WC_3bases sheet: CFA-broad / CFA-notes / SET side by side
- ทดสอบ notes parser ทุกบริษัท: เฉพาะ DUSIT parse สะอาด; MINT/SHANG/MANRIN/
  OHTL/SHR/VRANDA หมายเหตุคนละ format (หัวข้อ/หน่วย/โครงต่าง) -> อัตโนมัติครบ 10 ไม่ได้
- extract_notes: เพิ่ม unit detection (ล้านบาท/พันบาท), normalize เป็นล้านบาท
- trade_notes.csv: เก็บ DSO การค้าล้วนที่ verify แล้ว (DUSIT 20.7, MINT 26)
- report.py: ชีต WC_3bases แสดง DSO/DIO/DPO 3 ฐาน (CFA-broad ครบ10 /
  CFA-notes เฉพาะที่ดึงได้ / SET ครบ10)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WjBjdz26s52MeASaozo8gq
</commit_message>
<xml_diff>
--- a/tour-finance/output/ratios_report.xlsx
+++ b/tour-finance/output/ratios_report.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary_FY" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SET_vs_CFA" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WC_3bases" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External_MINT" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
@@ -963,7 +963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -972,7 +972,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DSO/DIO/DPO/CCC รายปี FY2568 — 2 ฐาน</t>
+          <t>วงจรเงินสดรายปี FY2568 — 3 ฐาน (DSO/DIO/DPO วัน)</t>
         </is>
       </c>
     </row>
@@ -980,20 +980,25 @@
       <c r="A2" s="3" t="inlineStr"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>SET basis (เทียบเว็บ)</t>
+          <t>CFA-broad (หน้างบดุล ครบ 10)</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr"/>
       <c r="D2" s="3" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr"/>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>CFA basis (ตามงบ)</t>
-        </is>
-      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>CFA-notes (การค้าล้วน)</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr"/>
       <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="3" t="inlineStr"/>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>SET (เทียบเว็บ)</t>
+        </is>
+      </c>
       <c r="I2" s="3" t="inlineStr"/>
+      <c r="J2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1018,27 +1023,32 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>CCC</t>
+          <t>DSO</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
+          <t>DIO</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>DPO</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
           <t>DSO</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>DIO</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>DPO</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>CCC</t>
         </is>
       </c>
     </row>
@@ -1049,28 +1059,22 @@
         </is>
       </c>
       <c r="B4" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="C4" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="D4" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="H4" t="n">
         <v>25.7</v>
       </c>
-      <c r="C4" t="n">
+      <c r="I4" t="n">
         <v>17.8</v>
       </c>
-      <c r="D4" t="n">
+      <c r="J4" t="n">
         <v>12.7</v>
-      </c>
-      <c r="E4" t="n">
-        <v>30.8</v>
-      </c>
-      <c r="F4" t="n">
-        <v>23.8</v>
-      </c>
-      <c r="G4" t="n">
-        <v>17.9</v>
-      </c>
-      <c r="H4" t="n">
-        <v>12.8</v>
-      </c>
-      <c r="I4" t="n">
-        <v>28.9</v>
       </c>
     </row>
     <row r="5">
@@ -1080,28 +1084,22 @@
         </is>
       </c>
       <c r="B5" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="C5" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>114.1</v>
+      </c>
+      <c r="H5" t="n">
         <v>14.7</v>
       </c>
-      <c r="C5" t="n">
+      <c r="I5" t="n">
         <v>23.7</v>
       </c>
-      <c r="D5" t="n">
+      <c r="J5" t="n">
         <v>116.3</v>
-      </c>
-      <c r="E5" t="n">
-        <v>-78</v>
-      </c>
-      <c r="F5" t="n">
-        <v>15.8</v>
-      </c>
-      <c r="G5" t="n">
-        <v>24.2</v>
-      </c>
-      <c r="H5" t="n">
-        <v>114.1</v>
-      </c>
-      <c r="I5" t="n">
-        <v>-74.09999999999999</v>
       </c>
     </row>
     <row r="6">
@@ -1111,28 +1109,25 @@
         </is>
       </c>
       <c r="B6" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="C6" t="n">
+        <v>9</v>
+      </c>
+      <c r="D6" t="n">
+        <v>135</v>
+      </c>
+      <c r="E6" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="H6" t="n">
         <v>68.40000000000001</v>
       </c>
-      <c r="C6" t="n">
+      <c r="I6" t="n">
         <v>9.1</v>
       </c>
-      <c r="D6" t="n">
+      <c r="J6" t="n">
         <v>181.6</v>
-      </c>
-      <c r="E6" t="n">
-        <v>-104.1</v>
-      </c>
-      <c r="F6" t="n">
-        <v>53.7</v>
-      </c>
-      <c r="G6" t="n">
-        <v>9</v>
-      </c>
-      <c r="H6" t="n">
-        <v>135</v>
-      </c>
-      <c r="I6" t="n">
-        <v>-72.3</v>
       </c>
     </row>
     <row r="7">
@@ -1142,28 +1137,22 @@
         </is>
       </c>
       <c r="B7" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="C7" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="D7" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="H7" t="n">
         <v>10.7</v>
       </c>
-      <c r="C7" t="n">
+      <c r="I7" t="n">
         <v>4.5</v>
       </c>
-      <c r="D7" t="n">
+      <c r="J7" t="n">
         <v>99.7</v>
-      </c>
-      <c r="E7" t="n">
-        <v>-84.40000000000001</v>
-      </c>
-      <c r="F7" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="G7" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="H7" t="n">
-        <v>29.3</v>
-      </c>
-      <c r="I7" t="n">
-        <v>-14.1</v>
       </c>
     </row>
     <row r="8">
@@ -1173,28 +1162,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10.7</v>
+        <v>12</v>
       </c>
       <c r="C8" t="n">
         <v>2.8</v>
       </c>
       <c r="D8" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="H8" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="I8" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="J8" t="n">
         <v>52</v>
-      </c>
-      <c r="E8" t="n">
-        <v>-38.5</v>
-      </c>
-      <c r="F8" t="n">
-        <v>12</v>
-      </c>
-      <c r="G8" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="H8" t="n">
-        <v>60.2</v>
-      </c>
-      <c r="I8" t="n">
-        <v>-45.4</v>
       </c>
     </row>
     <row r="9">
@@ -1204,28 +1187,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>36</v>
+        <v>32.9</v>
       </c>
       <c r="C9" t="n">
         <v>16.6</v>
       </c>
       <c r="D9" t="n">
+        <v>105.9</v>
+      </c>
+      <c r="E9" t="n">
+        <v>26</v>
+      </c>
+      <c r="H9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I9" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="J9" t="n">
         <v>143.6</v>
-      </c>
-      <c r="E9" t="n">
-        <v>-91.09999999999999</v>
-      </c>
-      <c r="F9" t="n">
-        <v>32.9</v>
-      </c>
-      <c r="G9" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="H9" t="n">
-        <v>105.9</v>
-      </c>
-      <c r="I9" t="n">
-        <v>-56.4</v>
       </c>
     </row>
     <row r="10">
@@ -1235,28 +1215,22 @@
         </is>
       </c>
       <c r="B10" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="C10" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="D10" t="n">
+        <v>133.3</v>
+      </c>
+      <c r="H10" t="n">
         <v>15.5</v>
       </c>
-      <c r="C10" t="n">
+      <c r="I10" t="n">
         <v>10</v>
       </c>
-      <c r="D10" t="n">
+      <c r="J10" t="n">
         <v>168</v>
-      </c>
-      <c r="E10" t="n">
-        <v>-142.5</v>
-      </c>
-      <c r="F10" t="n">
-        <v>13.8</v>
-      </c>
-      <c r="G10" t="n">
-        <v>8.9</v>
-      </c>
-      <c r="H10" t="n">
-        <v>133.3</v>
-      </c>
-      <c r="I10" t="n">
-        <v>-110.5</v>
       </c>
     </row>
     <row r="11">
@@ -1266,28 +1240,22 @@
         </is>
       </c>
       <c r="B11" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="C11" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="D11" t="n">
+        <v>129.7</v>
+      </c>
+      <c r="H11" t="n">
         <v>15.4</v>
       </c>
-      <c r="C11" t="n">
+      <c r="I11" t="n">
         <v>14.6</v>
       </c>
-      <c r="D11" t="n">
+      <c r="J11" t="n">
         <v>147.9</v>
-      </c>
-      <c r="E11" t="n">
-        <v>-117.8</v>
-      </c>
-      <c r="F11" t="n">
-        <v>14.4</v>
-      </c>
-      <c r="G11" t="n">
-        <v>14.9</v>
-      </c>
-      <c r="H11" t="n">
-        <v>129.7</v>
-      </c>
-      <c r="I11" t="n">
-        <v>-100.5</v>
       </c>
     </row>
     <row r="12">
@@ -1297,28 +1265,22 @@
         </is>
       </c>
       <c r="B12" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="C12" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="D12" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="H12" t="n">
         <v>14.4</v>
       </c>
-      <c r="C12" t="n">
+      <c r="I12" t="n">
         <v>14.2</v>
       </c>
-      <c r="D12" t="n">
+      <c r="J12" t="n">
         <v>71</v>
-      </c>
-      <c r="E12" t="n">
-        <v>-42.4</v>
-      </c>
-      <c r="F12" t="n">
-        <v>15.5</v>
-      </c>
-      <c r="G12" t="n">
-        <v>13.9</v>
-      </c>
-      <c r="H12" t="n">
-        <v>57.7</v>
-      </c>
-      <c r="I12" t="n">
-        <v>-28.4</v>
       </c>
     </row>
     <row r="13">
@@ -1328,28 +1290,43 @@
         </is>
       </c>
       <c r="B13" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="C13" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="D13" t="n">
+        <v>143.2</v>
+      </c>
+      <c r="H13" t="n">
         <v>12.6</v>
       </c>
-      <c r="C13" t="n">
+      <c r="I13" t="n">
         <v>8.6</v>
       </c>
-      <c r="D13" t="n">
+      <c r="J13" t="n">
         <v>104.3</v>
       </c>
-      <c r="E13" t="n">
-        <v>-83.09999999999999</v>
-      </c>
-      <c r="F13" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="G13" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="H13" t="n">
-        <v>143.2</v>
-      </c>
-      <c r="I13" t="n">
-        <v>-122.8</v>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>หมายเหตุ: CFA-broad=ลูกหนี้/เจ้าหนี้หน้างบดุล (การค้า+หมุนเวียนอื่น) นิยามเดียวครบ 10 บริษัท</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CFA-notes=การค้าล้วนจากหมายเหตุ — เฉพาะ DUSIT/MINT ที่ดึงได้สะอาด (verify ตรงบริษัท); บริษัทอื่นหมายเหตุคนละ format ต้อง hand-code รายเจ้า</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SET=สูตร settrade (ปลายงวด, รายได้ดำเนินงาน, เจ้าหนี้กว้าง)</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert "Add WC_3bases sheet: CFA-broad / CFA-notes / SET side by side"
This reverts commit be688f999b708bb105bbeb66a40b015fe38f02d8.
</commit_message>
<xml_diff>
--- a/tour-finance/output/ratios_report.xlsx
+++ b/tour-finance/output/ratios_report.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary_FY" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WC_3bases" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SET_vs_CFA" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External_MINT" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
@@ -963,7 +963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -972,7 +972,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>วงจรเงินสดรายปี FY2568 — 3 ฐาน (DSO/DIO/DPO วัน)</t>
+          <t>DSO/DIO/DPO/CCC รายปี FY2568 — 2 ฐาน</t>
         </is>
       </c>
     </row>
@@ -980,25 +980,20 @@
       <c r="A2" s="3" t="inlineStr"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>CFA-broad (หน้างบดุล ครบ 10)</t>
+          <t>SET basis (เทียบเว็บ)</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr"/>
       <c r="D2" s="3" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>CFA-notes (การค้าล้วน)</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="inlineStr"/>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>CFA basis (ตามงบ)</t>
+        </is>
+      </c>
       <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>SET (เทียบเว็บ)</t>
-        </is>
-      </c>
+      <c r="H2" s="3" t="inlineStr"/>
       <c r="I2" s="3" t="inlineStr"/>
-      <c r="J2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1023,32 +1018,27 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
+          <t>CCC</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>DSO</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>DIO</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>DPO</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>DSO</t>
-        </is>
-      </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>DIO</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>DPO</t>
+          <t>CCC</t>
         </is>
       </c>
     </row>
@@ -1059,22 +1049,28 @@
         </is>
       </c>
       <c r="B4" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="C4" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="D4" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="E4" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="F4" t="n">
         <v>23.8</v>
       </c>
-      <c r="C4" t="n">
+      <c r="G4" t="n">
         <v>17.9</v>
       </c>
-      <c r="D4" t="n">
+      <c r="H4" t="n">
         <v>12.8</v>
       </c>
-      <c r="H4" t="n">
-        <v>25.7</v>
-      </c>
       <c r="I4" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="J4" t="n">
-        <v>12.7</v>
+        <v>28.9</v>
       </c>
     </row>
     <row r="5">
@@ -1084,22 +1080,28 @@
         </is>
       </c>
       <c r="B5" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="C5" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="D5" t="n">
+        <v>116.3</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-78</v>
+      </c>
+      <c r="F5" t="n">
         <v>15.8</v>
       </c>
-      <c r="C5" t="n">
+      <c r="G5" t="n">
         <v>24.2</v>
       </c>
-      <c r="D5" t="n">
+      <c r="H5" t="n">
         <v>114.1</v>
       </c>
-      <c r="H5" t="n">
-        <v>14.7</v>
-      </c>
       <c r="I5" t="n">
-        <v>23.7</v>
-      </c>
-      <c r="J5" t="n">
-        <v>116.3</v>
+        <v>-74.09999999999999</v>
       </c>
     </row>
     <row r="6">
@@ -1109,25 +1111,28 @@
         </is>
       </c>
       <c r="B6" t="n">
+        <v>68.40000000000001</v>
+      </c>
+      <c r="C6" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>181.6</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-104.1</v>
+      </c>
+      <c r="F6" t="n">
         <v>53.7</v>
       </c>
-      <c r="C6" t="n">
+      <c r="G6" t="n">
         <v>9</v>
       </c>
-      <c r="D6" t="n">
+      <c r="H6" t="n">
         <v>135</v>
       </c>
-      <c r="E6" t="n">
-        <v>20.7</v>
-      </c>
-      <c r="H6" t="n">
-        <v>68.40000000000001</v>
-      </c>
       <c r="I6" t="n">
-        <v>9.1</v>
-      </c>
-      <c r="J6" t="n">
-        <v>181.6</v>
+        <v>-72.3</v>
       </c>
     </row>
     <row r="7">
@@ -1137,22 +1142,28 @@
         </is>
       </c>
       <c r="B7" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="C7" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D7" t="n">
+        <v>99.7</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-84.40000000000001</v>
+      </c>
+      <c r="F7" t="n">
         <v>10.5</v>
       </c>
-      <c r="C7" t="n">
+      <c r="G7" t="n">
         <v>4.7</v>
       </c>
-      <c r="D7" t="n">
+      <c r="H7" t="n">
         <v>29.3</v>
       </c>
-      <c r="H7" t="n">
-        <v>10.7</v>
-      </c>
       <c r="I7" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="J7" t="n">
-        <v>99.7</v>
+        <v>-14.1</v>
       </c>
     </row>
     <row r="8">
@@ -1162,22 +1173,28 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>12</v>
+        <v>10.7</v>
       </c>
       <c r="C8" t="n">
         <v>2.8</v>
       </c>
       <c r="D8" t="n">
+        <v>52</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-38.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>12</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="H8" t="n">
         <v>60.2</v>
       </c>
-      <c r="H8" t="n">
-        <v>10.7</v>
-      </c>
       <c r="I8" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="J8" t="n">
-        <v>52</v>
+        <v>-45.4</v>
       </c>
     </row>
     <row r="9">
@@ -1187,25 +1204,28 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>32.9</v>
+        <v>36</v>
       </c>
       <c r="C9" t="n">
         <v>16.6</v>
       </c>
       <c r="D9" t="n">
+        <v>143.6</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-91.09999999999999</v>
+      </c>
+      <c r="F9" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="G9" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="H9" t="n">
         <v>105.9</v>
       </c>
-      <c r="E9" t="n">
-        <v>26</v>
-      </c>
-      <c r="H9" t="n">
-        <v>36</v>
-      </c>
       <c r="I9" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="J9" t="n">
-        <v>143.6</v>
+        <v>-56.4</v>
       </c>
     </row>
     <row r="10">
@@ -1215,22 +1235,28 @@
         </is>
       </c>
       <c r="B10" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="C10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" t="n">
+        <v>168</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-142.5</v>
+      </c>
+      <c r="F10" t="n">
         <v>13.8</v>
       </c>
-      <c r="C10" t="n">
+      <c r="G10" t="n">
         <v>8.9</v>
       </c>
-      <c r="D10" t="n">
+      <c r="H10" t="n">
         <v>133.3</v>
       </c>
-      <c r="H10" t="n">
-        <v>15.5</v>
-      </c>
       <c r="I10" t="n">
-        <v>10</v>
-      </c>
-      <c r="J10" t="n">
-        <v>168</v>
+        <v>-110.5</v>
       </c>
     </row>
     <row r="11">
@@ -1240,22 +1266,28 @@
         </is>
       </c>
       <c r="B11" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="C11" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="D11" t="n">
+        <v>147.9</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-117.8</v>
+      </c>
+      <c r="F11" t="n">
         <v>14.4</v>
       </c>
-      <c r="C11" t="n">
+      <c r="G11" t="n">
         <v>14.9</v>
       </c>
-      <c r="D11" t="n">
+      <c r="H11" t="n">
         <v>129.7</v>
       </c>
-      <c r="H11" t="n">
-        <v>15.4</v>
-      </c>
       <c r="I11" t="n">
-        <v>14.6</v>
-      </c>
-      <c r="J11" t="n">
-        <v>147.9</v>
+        <v>-100.5</v>
       </c>
     </row>
     <row r="12">
@@ -1265,22 +1297,28 @@
         </is>
       </c>
       <c r="B12" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="C12" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="D12" t="n">
+        <v>71</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-42.4</v>
+      </c>
+      <c r="F12" t="n">
         <v>15.5</v>
       </c>
-      <c r="C12" t="n">
+      <c r="G12" t="n">
         <v>13.9</v>
       </c>
-      <c r="D12" t="n">
+      <c r="H12" t="n">
         <v>57.7</v>
       </c>
-      <c r="H12" t="n">
-        <v>14.4</v>
-      </c>
       <c r="I12" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="J12" t="n">
-        <v>71</v>
+        <v>-28.4</v>
       </c>
     </row>
     <row r="13">
@@ -1290,43 +1328,28 @@
         </is>
       </c>
       <c r="B13" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="C13" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="D13" t="n">
+        <v>104.3</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-83.09999999999999</v>
+      </c>
+      <c r="F13" t="n">
         <v>12.5</v>
       </c>
-      <c r="C13" t="n">
+      <c r="G13" t="n">
         <v>7.8</v>
       </c>
-      <c r="D13" t="n">
+      <c r="H13" t="n">
         <v>143.2</v>
       </c>
-      <c r="H13" t="n">
-        <v>12.6</v>
-      </c>
       <c r="I13" t="n">
-        <v>8.6</v>
-      </c>
-      <c r="J13" t="n">
-        <v>104.3</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>หมายเหตุ: CFA-broad=ลูกหนี้/เจ้าหนี้หน้างบดุล (การค้า+หมุนเวียนอื่น) นิยามเดียวครบ 10 บริษัท</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>CFA-notes=การค้าล้วนจากหมายเหตุ — เฉพาะ DUSIT/MINT ที่ดึงได้สะอาด (verify ตรงบริษัท); บริษัทอื่นหมายเหตุคนละ format ต้อง hand-code รายเจ้า</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>SET=สูตร settrade (ปลายงวด, รายได้ดำเนินงาน, เจ้าหนี้กว้าง)</t>
-        </is>
+        <v>-122.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add metrics_all.xlsx (200-point dataset, rev_low highlighted); refresh Excel deliverables
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WjBjdz26s52MeASaozo8gq
</commit_message>
<xml_diff>
--- a/tour-finance/output/ratios_report.xlsx
+++ b/tour-finance/output/ratios_report.xlsx
@@ -1781,7 +1781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U201"/>
+  <dimension ref="A1:V201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1885,10 +1885,15 @@
       </c>
       <c r="T1" s="2" t="inlineStr">
         <is>
+          <t>rev_low</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
           <t>balance_ok</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>source</t>
         </is>
@@ -1990,12 +1995,13 @@
           <t>90.3468</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>Q1_FS.xls</t>
         </is>
@@ -2097,12 +2103,13 @@
           <t>104.9533</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>Q2_FS.xls</t>
         </is>
@@ -2204,12 +2211,13 @@
           <t>121.8953</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>Q3_FS.xls</t>
         </is>
@@ -2313,6 +2321,7 @@
       </c>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2410,12 +2419,13 @@
           <t>84.9768</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>Q1_FS.xls</t>
         </is>
@@ -2517,12 +2527,13 @@
           <t>71.5805</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="V7" t="inlineStr">
         <is>
           <t>Q2_FS.xls</t>
         </is>
@@ -2624,12 +2635,13 @@
           <t>56.34</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>Q3_FS.xls</t>
         </is>
@@ -2733,6 +2745,7 @@
       </c>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2830,12 +2843,13 @@
           <t>49.1502</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="V10" t="inlineStr">
         <is>
           <t>Q1_FS.xls</t>
         </is>
@@ -2937,12 +2951,13 @@
           <t>52.4888</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr">
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="V11" t="inlineStr">
         <is>
           <t>Q2_FS.xls</t>
         </is>
@@ -3044,12 +3059,13 @@
           <t>50.1435</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="V12" t="inlineStr">
         <is>
           <t>Q3_FS.xls</t>
         </is>
@@ -3153,6 +3169,7 @@
       </c>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3250,12 +3267,13 @@
           <t>41.324</t>
         </is>
       </c>
-      <c r="T14" t="inlineStr">
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="V14" t="inlineStr">
         <is>
           <t>Q1_FS.xls</t>
         </is>
@@ -3357,12 +3375,13 @@
           <t>41.7304</t>
         </is>
       </c>
-      <c r="T15" t="inlineStr">
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
+      <c r="V15" t="inlineStr">
         <is>
           <t>Q2_FS.xls</t>
         </is>
@@ -3464,12 +3483,13 @@
           <t>36.1948</t>
         </is>
       </c>
-      <c r="T16" t="inlineStr">
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="V16" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -3573,6 +3593,7 @@
       </c>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3670,12 +3691,13 @@
           <t>27.6284</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr">
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
+      <c r="V18" t="inlineStr">
         <is>
           <t>Q1_FS.xls</t>
         </is>
@@ -3777,12 +3799,13 @@
           <t>30.5733</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr">
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="V19" t="inlineStr">
         <is>
           <t>Q2_FS.xls</t>
         </is>
@@ -3884,12 +3907,13 @@
           <t>31.439</t>
         </is>
       </c>
-      <c r="T20" t="inlineStr">
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
+      <c r="V20" t="inlineStr">
         <is>
           <t>Q3_FS.xls</t>
         </is>
@@ -3993,6 +4017,7 @@
       </c>
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4090,12 +4115,13 @@
           <t>-34.1986</t>
         </is>
       </c>
-      <c r="T22" t="inlineStr">
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr">
+      <c r="V22" t="inlineStr">
         <is>
           <t>Q1_FS.xls</t>
         </is>
@@ -4197,12 +4223,13 @@
           <t>-36.7226</t>
         </is>
       </c>
-      <c r="T23" t="inlineStr">
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr">
+      <c r="V23" t="inlineStr">
         <is>
           <t>Q2_FS.xls</t>
         </is>
@@ -4304,12 +4331,13 @@
           <t>-50.6431</t>
         </is>
       </c>
-      <c r="T24" t="inlineStr">
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr">
+      <c r="V24" t="inlineStr">
         <is>
           <t>Q3_FS.xls</t>
         </is>
@@ -4413,6 +4441,7 @@
       </c>
       <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4510,12 +4539,13 @@
           <t>-52.0574</t>
         </is>
       </c>
-      <c r="T26" t="inlineStr">
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
+      <c r="V26" t="inlineStr">
         <is>
           <t>Q1_FS.xls</t>
         </is>
@@ -4617,12 +4647,13 @@
           <t>-46.6762</t>
         </is>
       </c>
-      <c r="T27" t="inlineStr">
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U27" t="inlineStr">
+      <c r="V27" t="inlineStr">
         <is>
           <t>Q2_FS.xls</t>
         </is>
@@ -4724,12 +4755,13 @@
           <t>-50.1574</t>
         </is>
       </c>
-      <c r="T28" t="inlineStr">
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U28" t="inlineStr">
+      <c r="V28" t="inlineStr">
         <is>
           <t>Q3_FS.xls</t>
         </is>
@@ -4833,6 +4865,7 @@
       </c>
       <c r="T29" t="inlineStr"/>
       <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4930,12 +4963,13 @@
           <t>-48.5433</t>
         </is>
       </c>
-      <c r="T30" t="inlineStr">
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U30" t="inlineStr">
+      <c r="V30" t="inlineStr">
         <is>
           <t>Q1_FS.xls</t>
         </is>
@@ -5037,12 +5071,13 @@
           <t>-39.2266</t>
         </is>
       </c>
-      <c r="T31" t="inlineStr">
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U31" t="inlineStr">
+      <c r="V31" t="inlineStr">
         <is>
           <t>Q2_FS.xls</t>
         </is>
@@ -5144,12 +5179,13 @@
           <t>-35.557</t>
         </is>
       </c>
-      <c r="T32" t="inlineStr">
+      <c r="T32" t="inlineStr"/>
+      <c r="U32" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr">
+      <c r="V32" t="inlineStr">
         <is>
           <t>Q3_FS.xls</t>
         </is>
@@ -5253,6 +5289,7 @@
       </c>
       <c r="T33" t="inlineStr"/>
       <c r="U33" t="inlineStr"/>
+      <c r="V33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5350,12 +5387,13 @@
           <t>-41.5612</t>
         </is>
       </c>
-      <c r="T34" t="inlineStr">
+      <c r="T34" t="inlineStr"/>
+      <c r="U34" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U34" t="inlineStr">
+      <c r="V34" t="inlineStr">
         <is>
           <t>Q1_FS.xls</t>
         </is>
@@ -5457,12 +5495,13 @@
           <t>-48.2738</t>
         </is>
       </c>
-      <c r="T35" t="inlineStr">
+      <c r="T35" t="inlineStr"/>
+      <c r="U35" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U35" t="inlineStr">
+      <c r="V35" t="inlineStr">
         <is>
           <t>Q2_FS.xls</t>
         </is>
@@ -5564,12 +5603,13 @@
           <t>-59.7923</t>
         </is>
       </c>
-      <c r="T36" t="inlineStr">
+      <c r="T36" t="inlineStr"/>
+      <c r="U36" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U36" t="inlineStr">
+      <c r="V36" t="inlineStr">
         <is>
           <t>Q3_FS.xls</t>
         </is>
@@ -5673,6 +5713,7 @@
       </c>
       <c r="T37" t="inlineStr"/>
       <c r="U37" t="inlineStr"/>
+      <c r="V37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5770,12 +5811,13 @@
           <t>-63.8475</t>
         </is>
       </c>
-      <c r="T38" t="inlineStr">
+      <c r="T38" t="inlineStr"/>
+      <c r="U38" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U38" t="inlineStr">
+      <c r="V38" t="inlineStr">
         <is>
           <t>Q1_FS.xls</t>
         </is>
@@ -5877,12 +5919,13 @@
           <t>-50.0908</t>
         </is>
       </c>
-      <c r="T39" t="inlineStr">
+      <c r="T39" t="inlineStr"/>
+      <c r="U39" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U39" t="inlineStr">
+      <c r="V39" t="inlineStr">
         <is>
           <t>Q2_FS.xls</t>
         </is>
@@ -5984,12 +6027,13 @@
           <t>-56.3605</t>
         </is>
       </c>
-      <c r="T40" t="inlineStr">
+      <c r="T40" t="inlineStr"/>
+      <c r="U40" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U40" t="inlineStr">
+      <c r="V40" t="inlineStr">
         <is>
           <t>Q3_FS.xls</t>
         </is>
@@ -6093,6 +6137,7 @@
       </c>
       <c r="T41" t="inlineStr"/>
       <c r="U41" t="inlineStr"/>
+      <c r="V41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -6190,12 +6235,13 @@
           <t>-138.4739</t>
         </is>
       </c>
-      <c r="T42" t="inlineStr">
+      <c r="T42" t="inlineStr"/>
+      <c r="U42" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U42" t="inlineStr">
+      <c r="V42" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -6297,12 +6343,13 @@
           <t>-206.4327</t>
         </is>
       </c>
-      <c r="T43" t="inlineStr">
+      <c r="T43" t="inlineStr"/>
+      <c r="U43" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U43" t="inlineStr">
+      <c r="V43" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -6404,12 +6451,13 @@
           <t>-149.5471</t>
         </is>
       </c>
-      <c r="T44" t="inlineStr">
+      <c r="T44" t="inlineStr"/>
+      <c r="U44" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U44" t="inlineStr">
+      <c r="V44" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -6513,6 +6561,7 @@
       </c>
       <c r="T45" t="inlineStr"/>
       <c r="U45" t="inlineStr"/>
+      <c r="V45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -6610,12 +6659,13 @@
           <t>-121.4683</t>
         </is>
       </c>
-      <c r="T46" t="inlineStr">
+      <c r="T46" t="inlineStr"/>
+      <c r="U46" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U46" t="inlineStr">
+      <c r="V46" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -6717,12 +6767,13 @@
           <t>-124.8645</t>
         </is>
       </c>
-      <c r="T47" t="inlineStr">
+      <c r="T47" t="inlineStr"/>
+      <c r="U47" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U47" t="inlineStr">
+      <c r="V47" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -6824,12 +6875,13 @@
           <t>-134.0293</t>
         </is>
       </c>
-      <c r="T48" t="inlineStr">
+      <c r="T48" t="inlineStr"/>
+      <c r="U48" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U48" t="inlineStr">
+      <c r="V48" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -6933,6 +6985,7 @@
       </c>
       <c r="T49" t="inlineStr"/>
       <c r="U49" t="inlineStr"/>
+      <c r="V49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -7030,12 +7083,13 @@
           <t>-135.334</t>
         </is>
       </c>
-      <c r="T50" t="inlineStr">
+      <c r="T50" t="inlineStr"/>
+      <c r="U50" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U50" t="inlineStr">
+      <c r="V50" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -7137,12 +7191,13 @@
           <t>-136.2981</t>
         </is>
       </c>
-      <c r="T51" t="inlineStr">
+      <c r="T51" t="inlineStr"/>
+      <c r="U51" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U51" t="inlineStr">
+      <c r="V51" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -7244,12 +7299,13 @@
           <t>-123.6786</t>
         </is>
       </c>
-      <c r="T52" t="inlineStr">
+      <c r="T52" t="inlineStr"/>
+      <c r="U52" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U52" t="inlineStr">
+      <c r="V52" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -7353,6 +7409,7 @@
       </c>
       <c r="T53" t="inlineStr"/>
       <c r="U53" t="inlineStr"/>
+      <c r="V53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -7450,12 +7507,13 @@
           <t>-123.1863</t>
         </is>
       </c>
-      <c r="T54" t="inlineStr">
+      <c r="T54" t="inlineStr"/>
+      <c r="U54" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U54" t="inlineStr">
+      <c r="V54" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -7557,12 +7615,13 @@
           <t>-146.1746</t>
         </is>
       </c>
-      <c r="T55" t="inlineStr">
+      <c r="T55" t="inlineStr"/>
+      <c r="U55" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U55" t="inlineStr">
+      <c r="V55" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -7664,12 +7723,13 @@
           <t>-132.3507</t>
         </is>
       </c>
-      <c r="T56" t="inlineStr">
+      <c r="T56" t="inlineStr"/>
+      <c r="U56" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U56" t="inlineStr">
+      <c r="V56" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -7773,6 +7833,7 @@
       </c>
       <c r="T57" t="inlineStr"/>
       <c r="U57" t="inlineStr"/>
+      <c r="V57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -7870,12 +7931,13 @@
           <t>-75.5416</t>
         </is>
       </c>
-      <c r="T58" t="inlineStr">
+      <c r="T58" t="inlineStr"/>
+      <c r="U58" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U58" t="inlineStr">
+      <c r="V58" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -7977,12 +8039,13 @@
           <t>-79.3769</t>
         </is>
       </c>
-      <c r="T59" t="inlineStr">
+      <c r="T59" t="inlineStr"/>
+      <c r="U59" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U59" t="inlineStr">
+      <c r="V59" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -8084,12 +8147,13 @@
           <t>-69.9465</t>
         </is>
       </c>
-      <c r="T60" t="inlineStr">
+      <c r="T60" t="inlineStr"/>
+      <c r="U60" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U60" t="inlineStr">
+      <c r="V60" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -8193,6 +8257,7 @@
       </c>
       <c r="T61" t="inlineStr"/>
       <c r="U61" t="inlineStr"/>
+      <c r="V61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -8292,10 +8357,15 @@
       </c>
       <c r="T62" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U62" t="inlineStr">
+      <c r="V62" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -8399,10 +8469,15 @@
       </c>
       <c r="T63" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U63" t="inlineStr">
+      <c r="V63" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -8506,10 +8581,15 @@
       </c>
       <c r="T64" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U64" t="inlineStr">
+      <c r="V64" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -8613,6 +8693,7 @@
       </c>
       <c r="T65" t="inlineStr"/>
       <c r="U65" t="inlineStr"/>
+      <c r="V65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -8712,10 +8793,15 @@
       </c>
       <c r="T66" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U66" t="inlineStr">
+      <c r="V66" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -8817,12 +8903,13 @@
           <t>-3.5416</t>
         </is>
       </c>
-      <c r="T67" t="inlineStr">
+      <c r="T67" t="inlineStr"/>
+      <c r="U67" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U67" t="inlineStr">
+      <c r="V67" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -8924,12 +9011,13 @@
           <t>-5.3394</t>
         </is>
       </c>
-      <c r="T68" t="inlineStr">
+      <c r="T68" t="inlineStr"/>
+      <c r="U68" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U68" t="inlineStr">
+      <c r="V68" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -9033,6 +9121,7 @@
       </c>
       <c r="T69" t="inlineStr"/>
       <c r="U69" t="inlineStr"/>
+      <c r="V69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -9130,12 +9219,13 @@
           <t>-11.0043</t>
         </is>
       </c>
-      <c r="T70" t="inlineStr">
+      <c r="T70" t="inlineStr"/>
+      <c r="U70" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U70" t="inlineStr">
+      <c r="V70" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -9237,12 +9327,13 @@
           <t>-7.7003</t>
         </is>
       </c>
-      <c r="T71" t="inlineStr">
+      <c r="T71" t="inlineStr"/>
+      <c r="U71" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U71" t="inlineStr">
+      <c r="V71" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -9344,12 +9435,13 @@
           <t>-8.5235</t>
         </is>
       </c>
-      <c r="T72" t="inlineStr">
+      <c r="T72" t="inlineStr"/>
+      <c r="U72" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U72" t="inlineStr">
+      <c r="V72" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -9453,6 +9545,7 @@
       </c>
       <c r="T73" t="inlineStr"/>
       <c r="U73" t="inlineStr"/>
+      <c r="V73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -9550,12 +9643,13 @@
           <t>-12.7501</t>
         </is>
       </c>
-      <c r="T74" t="inlineStr">
+      <c r="T74" t="inlineStr"/>
+      <c r="U74" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U74" t="inlineStr">
+      <c r="V74" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -9657,12 +9751,13 @@
           <t>-10.6574</t>
         </is>
       </c>
-      <c r="T75" t="inlineStr">
+      <c r="T75" t="inlineStr"/>
+      <c r="U75" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U75" t="inlineStr">
+      <c r="V75" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -9764,12 +9859,13 @@
           <t>-8.8176</t>
         </is>
       </c>
-      <c r="T76" t="inlineStr">
+      <c r="T76" t="inlineStr"/>
+      <c r="U76" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U76" t="inlineStr">
+      <c r="V76" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -9873,6 +9969,7 @@
       </c>
       <c r="T77" t="inlineStr"/>
       <c r="U77" t="inlineStr"/>
+      <c r="V77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -9970,12 +10067,13 @@
           <t>-11.145</t>
         </is>
       </c>
-      <c r="T78" t="inlineStr">
+      <c r="T78" t="inlineStr"/>
+      <c r="U78" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U78" t="inlineStr">
+      <c r="V78" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -10077,12 +10175,13 @@
           <t>-6.9673</t>
         </is>
       </c>
-      <c r="T79" t="inlineStr">
+      <c r="T79" t="inlineStr"/>
+      <c r="U79" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U79" t="inlineStr">
+      <c r="V79" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -10184,12 +10283,13 @@
           <t>-7.3971</t>
         </is>
       </c>
-      <c r="T80" t="inlineStr">
+      <c r="T80" t="inlineStr"/>
+      <c r="U80" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U80" t="inlineStr">
+      <c r="V80" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -10293,6 +10393,7 @@
       </c>
       <c r="T81" t="inlineStr"/>
       <c r="U81" t="inlineStr"/>
+      <c r="V81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -10392,10 +10493,15 @@
       </c>
       <c r="T82" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr">
+        <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U82" t="inlineStr">
+      <c r="V82" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -10499,10 +10605,15 @@
       </c>
       <c r="T83" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="U83" t="inlineStr">
+        <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U83" t="inlineStr">
+      <c r="V83" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -10606,10 +10717,15 @@
       </c>
       <c r="T84" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="U84" t="inlineStr">
+        <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U84" t="inlineStr">
+      <c r="V84" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -10713,10 +10829,15 @@
       </c>
       <c r="T85" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="U85" t="inlineStr">
+        <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U85" t="inlineStr">
+      <c r="V85" t="inlineStr">
         <is>
           <t>Q4_FS.xlsx</t>
         </is>
@@ -10820,10 +10941,15 @@
       </c>
       <c r="T86" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="U86" t="inlineStr">
+        <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U86" t="inlineStr">
+      <c r="V86" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -10925,12 +11051,13 @@
           <t>-26.4969</t>
         </is>
       </c>
-      <c r="T87" t="inlineStr">
+      <c r="T87" t="inlineStr"/>
+      <c r="U87" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U87" t="inlineStr">
+      <c r="V87" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -11032,12 +11159,13 @@
           <t>-37.8641</t>
         </is>
       </c>
-      <c r="T88" t="inlineStr">
+      <c r="T88" t="inlineStr"/>
+      <c r="U88" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U88" t="inlineStr">
+      <c r="V88" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -11139,12 +11267,13 @@
           <t>-44.9112</t>
         </is>
       </c>
-      <c r="T89" t="inlineStr">
+      <c r="T89" t="inlineStr"/>
+      <c r="U89" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U89" t="inlineStr">
+      <c r="V89" t="inlineStr">
         <is>
           <t>Q4_FS.xlsx</t>
         </is>
@@ -11246,12 +11375,13 @@
           <t>-36.0845</t>
         </is>
       </c>
-      <c r="T90" t="inlineStr">
+      <c r="T90" t="inlineStr"/>
+      <c r="U90" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U90" t="inlineStr">
+      <c r="V90" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -11353,12 +11483,13 @@
           <t>-33.9583</t>
         </is>
       </c>
-      <c r="T91" t="inlineStr">
+      <c r="T91" t="inlineStr"/>
+      <c r="U91" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U91" t="inlineStr">
+      <c r="V91" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -11460,12 +11591,13 @@
           <t>-29.8926</t>
         </is>
       </c>
-      <c r="T92" t="inlineStr">
+      <c r="T92" t="inlineStr"/>
+      <c r="U92" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U92" t="inlineStr">
+      <c r="V92" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -11567,12 +11699,13 @@
           <t>-32.4413</t>
         </is>
       </c>
-      <c r="T93" t="inlineStr">
+      <c r="T93" t="inlineStr"/>
+      <c r="U93" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U93" t="inlineStr">
+      <c r="V93" t="inlineStr">
         <is>
           <t>Q4_FS.xlsx</t>
         </is>
@@ -11674,12 +11807,13 @@
           <t>-35.2182</t>
         </is>
       </c>
-      <c r="T94" t="inlineStr">
+      <c r="T94" t="inlineStr"/>
+      <c r="U94" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U94" t="inlineStr">
+      <c r="V94" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -11781,12 +11915,13 @@
           <t>-46.6039</t>
         </is>
       </c>
-      <c r="T95" t="inlineStr">
+      <c r="T95" t="inlineStr"/>
+      <c r="U95" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U95" t="inlineStr">
+      <c r="V95" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -11888,12 +12023,13 @@
           <t>-44.2165</t>
         </is>
       </c>
-      <c r="T96" t="inlineStr">
+      <c r="T96" t="inlineStr"/>
+      <c r="U96" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U96" t="inlineStr">
+      <c r="V96" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -11997,6 +12133,7 @@
       </c>
       <c r="T97" t="inlineStr"/>
       <c r="U97" t="inlineStr"/>
+      <c r="V97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -12094,12 +12231,13 @@
           <t>-43.3141</t>
         </is>
       </c>
-      <c r="T98" t="inlineStr">
+      <c r="T98" t="inlineStr"/>
+      <c r="U98" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U98" t="inlineStr">
+      <c r="V98" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -12201,12 +12339,13 @@
           <t>-38.3298</t>
         </is>
       </c>
-      <c r="T99" t="inlineStr">
+      <c r="T99" t="inlineStr"/>
+      <c r="U99" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U99" t="inlineStr">
+      <c r="V99" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -12308,12 +12447,13 @@
           <t>-41.447</t>
         </is>
       </c>
-      <c r="T100" t="inlineStr">
+      <c r="T100" t="inlineStr"/>
+      <c r="U100" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U100" t="inlineStr">
+      <c r="V100" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -12417,6 +12557,7 @@
       </c>
       <c r="T101" t="inlineStr"/>
       <c r="U101" t="inlineStr"/>
+      <c r="V101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -12516,10 +12657,15 @@
       </c>
       <c r="T102" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="U102" t="inlineStr">
+        <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U102" t="inlineStr">
+      <c r="V102" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -12621,12 +12767,13 @@
           <t>-39.4862</t>
         </is>
       </c>
-      <c r="T103" t="inlineStr">
+      <c r="T103" t="inlineStr"/>
+      <c r="U103" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U103" t="inlineStr">
+      <c r="V103" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -12728,12 +12875,13 @@
           <t>-43.0169</t>
         </is>
       </c>
-      <c r="T104" t="inlineStr">
+      <c r="T104" t="inlineStr"/>
+      <c r="U104" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U104" t="inlineStr">
+      <c r="V104" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -12837,6 +12985,7 @@
       </c>
       <c r="T105" t="inlineStr"/>
       <c r="U105" t="inlineStr"/>
+      <c r="V105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -12934,12 +13083,13 @@
           <t>-30.0101</t>
         </is>
       </c>
-      <c r="T106" t="inlineStr">
+      <c r="T106" t="inlineStr"/>
+      <c r="U106" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U106" t="inlineStr">
+      <c r="V106" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -13041,12 +13191,13 @@
           <t>-35.2856</t>
         </is>
       </c>
-      <c r="T107" t="inlineStr">
+      <c r="T107" t="inlineStr"/>
+      <c r="U107" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U107" t="inlineStr">
+      <c r="V107" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -13148,12 +13299,13 @@
           <t>-38.123</t>
         </is>
       </c>
-      <c r="T108" t="inlineStr">
+      <c r="T108" t="inlineStr"/>
+      <c r="U108" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U108" t="inlineStr">
+      <c r="V108" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -13257,6 +13409,7 @@
       </c>
       <c r="T109" t="inlineStr"/>
       <c r="U109" t="inlineStr"/>
+      <c r="V109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -13354,12 +13507,13 @@
           <t>-44.3549</t>
         </is>
       </c>
-      <c r="T110" t="inlineStr">
+      <c r="T110" t="inlineStr"/>
+      <c r="U110" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U110" t="inlineStr">
+      <c r="V110" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -13461,12 +13615,13 @@
           <t>-46.2404</t>
         </is>
       </c>
-      <c r="T111" t="inlineStr">
+      <c r="T111" t="inlineStr"/>
+      <c r="U111" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U111" t="inlineStr">
+      <c r="V111" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -13568,12 +13723,13 @@
           <t>-47.723</t>
         </is>
       </c>
-      <c r="T112" t="inlineStr">
+      <c r="T112" t="inlineStr"/>
+      <c r="U112" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U112" t="inlineStr">
+      <c r="V112" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -13677,6 +13833,7 @@
       </c>
       <c r="T113" t="inlineStr"/>
       <c r="U113" t="inlineStr"/>
+      <c r="V113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -13774,12 +13931,13 @@
           <t>-48.1028</t>
         </is>
       </c>
-      <c r="T114" t="inlineStr">
+      <c r="T114" t="inlineStr"/>
+      <c r="U114" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U114" t="inlineStr">
+      <c r="V114" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -13881,12 +14039,13 @@
           <t>-41.2806</t>
         </is>
       </c>
-      <c r="T115" t="inlineStr">
+      <c r="T115" t="inlineStr"/>
+      <c r="U115" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U115" t="inlineStr">
+      <c r="V115" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -13988,12 +14147,13 @@
           <t>-40.4259</t>
         </is>
       </c>
-      <c r="T116" t="inlineStr">
+      <c r="T116" t="inlineStr"/>
+      <c r="U116" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U116" t="inlineStr">
+      <c r="V116" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -14097,6 +14257,7 @@
       </c>
       <c r="T117" t="inlineStr"/>
       <c r="U117" t="inlineStr"/>
+      <c r="V117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -14194,12 +14355,13 @@
           <t>-51.5836</t>
         </is>
       </c>
-      <c r="T118" t="inlineStr">
+      <c r="T118" t="inlineStr"/>
+      <c r="U118" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U118" t="inlineStr">
+      <c r="V118" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -14301,12 +14463,13 @@
           <t>-46.9784</t>
         </is>
       </c>
-      <c r="T119" t="inlineStr">
+      <c r="T119" t="inlineStr"/>
+      <c r="U119" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U119" t="inlineStr">
+      <c r="V119" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -14408,12 +14571,13 @@
           <t>-47.2561</t>
         </is>
       </c>
-      <c r="T120" t="inlineStr">
+      <c r="T120" t="inlineStr"/>
+      <c r="U120" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U120" t="inlineStr">
+      <c r="V120" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -14517,6 +14681,7 @@
       </c>
       <c r="T121" t="inlineStr"/>
       <c r="U121" t="inlineStr"/>
+      <c r="V121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -14616,10 +14781,15 @@
       </c>
       <c r="T122" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="U122" t="inlineStr">
+        <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U122" t="inlineStr">
+      <c r="V122" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -14723,10 +14893,15 @@
       </c>
       <c r="T123" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="U123" t="inlineStr">
+        <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U123" t="inlineStr">
+      <c r="V123" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -14830,10 +15005,15 @@
       </c>
       <c r="T124" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="U124" t="inlineStr">
+        <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U124" t="inlineStr">
+      <c r="V124" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -14937,6 +15117,7 @@
       </c>
       <c r="T125" t="inlineStr"/>
       <c r="U125" t="inlineStr"/>
+      <c r="V125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -15034,12 +15215,13 @@
           <t>-80.3027</t>
         </is>
       </c>
-      <c r="T126" t="inlineStr">
+      <c r="T126" t="inlineStr"/>
+      <c r="U126" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U126" t="inlineStr">
+      <c r="V126" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -15141,12 +15323,13 @@
           <t>-68.8228</t>
         </is>
       </c>
-      <c r="T127" t="inlineStr">
+      <c r="T127" t="inlineStr"/>
+      <c r="U127" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U127" t="inlineStr">
+      <c r="V127" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -15248,12 +15431,13 @@
           <t>-64.3268</t>
         </is>
       </c>
-      <c r="T128" t="inlineStr">
+      <c r="T128" t="inlineStr"/>
+      <c r="U128" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U128" t="inlineStr">
+      <c r="V128" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -15357,6 +15541,7 @@
       </c>
       <c r="T129" t="inlineStr"/>
       <c r="U129" t="inlineStr"/>
+      <c r="V129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -15454,12 +15639,13 @@
           <t>-61.6328</t>
         </is>
       </c>
-      <c r="T130" t="inlineStr">
+      <c r="T130" t="inlineStr"/>
+      <c r="U130" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U130" t="inlineStr">
+      <c r="V130" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -15561,12 +15747,13 @@
           <t>-55.2913</t>
         </is>
       </c>
-      <c r="T131" t="inlineStr">
+      <c r="T131" t="inlineStr"/>
+      <c r="U131" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U131" t="inlineStr">
+      <c r="V131" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -15668,12 +15855,13 @@
           <t>-59.7513</t>
         </is>
       </c>
-      <c r="T132" t="inlineStr">
+      <c r="T132" t="inlineStr"/>
+      <c r="U132" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U132" t="inlineStr">
+      <c r="V132" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -15777,6 +15965,7 @@
       </c>
       <c r="T133" t="inlineStr"/>
       <c r="U133" t="inlineStr"/>
+      <c r="V133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -15874,12 +16063,13 @@
           <t>-70.4343</t>
         </is>
       </c>
-      <c r="T134" t="inlineStr">
+      <c r="T134" t="inlineStr"/>
+      <c r="U134" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U134" t="inlineStr">
+      <c r="V134" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -15981,12 +16171,13 @@
           <t>-69.4198</t>
         </is>
       </c>
-      <c r="T135" t="inlineStr">
+      <c r="T135" t="inlineStr"/>
+      <c r="U135" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U135" t="inlineStr">
+      <c r="V135" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -16088,12 +16279,13 @@
           <t>-60.4943</t>
         </is>
       </c>
-      <c r="T136" t="inlineStr">
+      <c r="T136" t="inlineStr"/>
+      <c r="U136" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U136" t="inlineStr">
+      <c r="V136" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -16197,6 +16389,7 @@
       </c>
       <c r="T137" t="inlineStr"/>
       <c r="U137" t="inlineStr"/>
+      <c r="V137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -16294,12 +16487,13 @@
           <t>-70.0614</t>
         </is>
       </c>
-      <c r="T138" t="inlineStr">
+      <c r="T138" t="inlineStr"/>
+      <c r="U138" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U138" t="inlineStr">
+      <c r="V138" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -16401,12 +16595,13 @@
           <t>-65.3703</t>
         </is>
       </c>
-      <c r="T139" t="inlineStr">
+      <c r="T139" t="inlineStr"/>
+      <c r="U139" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U139" t="inlineStr">
+      <c r="V139" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -16508,12 +16703,13 @@
           <t>-87.4455</t>
         </is>
       </c>
-      <c r="T140" t="inlineStr">
+      <c r="T140" t="inlineStr"/>
+      <c r="U140" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U140" t="inlineStr">
+      <c r="V140" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -16617,6 +16813,7 @@
       </c>
       <c r="T141" t="inlineStr"/>
       <c r="U141" t="inlineStr"/>
+      <c r="V141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -16716,10 +16913,15 @@
       </c>
       <c r="T142" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="U142" t="inlineStr">
+        <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U142" t="inlineStr">
+      <c r="V142" t="inlineStr">
         <is>
           <t>Q1_FS.xls</t>
         </is>
@@ -16823,10 +17025,15 @@
       </c>
       <c r="T143" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="U143" t="inlineStr">
+        <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U143" t="inlineStr">
+      <c r="V143" t="inlineStr">
         <is>
           <t>Q2_FS.xls</t>
         </is>
@@ -16930,10 +17137,15 @@
       </c>
       <c r="T144" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="U144" t="inlineStr">
+        <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U144" t="inlineStr">
+      <c r="V144" t="inlineStr">
         <is>
           <t>Q3_FS.xls</t>
         </is>
@@ -17035,8 +17247,13 @@
           <t>-62.3963</t>
         </is>
       </c>
-      <c r="T145" t="inlineStr"/>
+      <c r="T145" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="U145" t="inlineStr"/>
+      <c r="V145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -17136,10 +17353,15 @@
       </c>
       <c r="T146" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="U146" t="inlineStr">
+        <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U146" t="inlineStr">
+      <c r="V146" t="inlineStr">
         <is>
           <t>Q1_FS.xls</t>
         </is>
@@ -17241,12 +17463,13 @@
           <t>-53.0438</t>
         </is>
       </c>
-      <c r="T147" t="inlineStr">
+      <c r="T147" t="inlineStr"/>
+      <c r="U147" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U147" t="inlineStr">
+      <c r="V147" t="inlineStr">
         <is>
           <t>Q2_FS.xls</t>
         </is>
@@ -17348,12 +17571,13 @@
           <t>-44.6662</t>
         </is>
       </c>
-      <c r="T148" t="inlineStr">
+      <c r="T148" t="inlineStr"/>
+      <c r="U148" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U148" t="inlineStr">
+      <c r="V148" t="inlineStr">
         <is>
           <t>Q3_FS.xls</t>
         </is>
@@ -17457,6 +17681,7 @@
       </c>
       <c r="T149" t="inlineStr"/>
       <c r="U149" t="inlineStr"/>
+      <c r="V149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -17554,12 +17779,13 @@
           <t>-67.7888</t>
         </is>
       </c>
-      <c r="T150" t="inlineStr">
+      <c r="T150" t="inlineStr"/>
+      <c r="U150" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U150" t="inlineStr">
+      <c r="V150" t="inlineStr">
         <is>
           <t>Q1_FS.xls</t>
         </is>
@@ -17661,12 +17887,13 @@
           <t>-67.1399</t>
         </is>
       </c>
-      <c r="T151" t="inlineStr">
+      <c r="T151" t="inlineStr"/>
+      <c r="U151" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U151" t="inlineStr">
+      <c r="V151" t="inlineStr">
         <is>
           <t>Q2_FS.xls</t>
         </is>
@@ -17768,12 +17995,13 @@
           <t>-55.1688</t>
         </is>
       </c>
-      <c r="T152" t="inlineStr">
+      <c r="T152" t="inlineStr"/>
+      <c r="U152" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U152" t="inlineStr">
+      <c r="V152" t="inlineStr">
         <is>
           <t>Q3_FS.xls</t>
         </is>
@@ -17877,6 +18105,7 @@
       </c>
       <c r="T153" t="inlineStr"/>
       <c r="U153" t="inlineStr"/>
+      <c r="V153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -17974,12 +18203,13 @@
           <t>-71.1698</t>
         </is>
       </c>
-      <c r="T154" t="inlineStr">
+      <c r="T154" t="inlineStr"/>
+      <c r="U154" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U154" t="inlineStr">
+      <c r="V154" t="inlineStr">
         <is>
           <t>Q1_FS.xls</t>
         </is>
@@ -18081,12 +18311,13 @@
           <t>-73.5054</t>
         </is>
       </c>
-      <c r="T155" t="inlineStr">
+      <c r="T155" t="inlineStr"/>
+      <c r="U155" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U155" t="inlineStr">
+      <c r="V155" t="inlineStr">
         <is>
           <t>Q2_FS.xls</t>
         </is>
@@ -18188,12 +18419,13 @@
           <t>-61.4617</t>
         </is>
       </c>
-      <c r="T156" t="inlineStr">
+      <c r="T156" t="inlineStr"/>
+      <c r="U156" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U156" t="inlineStr">
+      <c r="V156" t="inlineStr">
         <is>
           <t>Q3_FS.xls</t>
         </is>
@@ -18297,6 +18529,7 @@
       </c>
       <c r="T157" t="inlineStr"/>
       <c r="U157" t="inlineStr"/>
+      <c r="V157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -18394,12 +18627,13 @@
           <t>-71.6747</t>
         </is>
       </c>
-      <c r="T158" t="inlineStr">
+      <c r="T158" t="inlineStr"/>
+      <c r="U158" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U158" t="inlineStr">
+      <c r="V158" t="inlineStr">
         <is>
           <t>Q1_FS.xls</t>
         </is>
@@ -18501,12 +18735,13 @@
           <t>-64.4845</t>
         </is>
       </c>
-      <c r="T159" t="inlineStr">
+      <c r="T159" t="inlineStr"/>
+      <c r="U159" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U159" t="inlineStr">
+      <c r="V159" t="inlineStr">
         <is>
           <t>Q2_FS.xls</t>
         </is>
@@ -18608,12 +18843,13 @@
           <t>-49.798</t>
         </is>
       </c>
-      <c r="T160" t="inlineStr">
+      <c r="T160" t="inlineStr"/>
+      <c r="U160" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U160" t="inlineStr">
+      <c r="V160" t="inlineStr">
         <is>
           <t>Q3_FS.xls</t>
         </is>
@@ -18717,6 +18953,7 @@
       </c>
       <c r="T161" t="inlineStr"/>
       <c r="U161" t="inlineStr"/>
+      <c r="V161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -18816,10 +19053,15 @@
       </c>
       <c r="T162" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="U162" t="inlineStr">
+        <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U162" t="inlineStr">
+      <c r="V162" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -18923,10 +19165,15 @@
       </c>
       <c r="T163" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="U163" t="inlineStr">
+        <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U163" t="inlineStr">
+      <c r="V163" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -19028,12 +19275,13 @@
           <t>-101.4784</t>
         </is>
       </c>
-      <c r="T164" t="inlineStr">
+      <c r="T164" t="inlineStr"/>
+      <c r="U164" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U164" t="inlineStr">
+      <c r="V164" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -19137,6 +19385,7 @@
       </c>
       <c r="T165" t="inlineStr"/>
       <c r="U165" t="inlineStr"/>
+      <c r="V165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -19234,12 +19483,13 @@
           <t>-81.118</t>
         </is>
       </c>
-      <c r="T166" t="inlineStr">
+      <c r="T166" t="inlineStr"/>
+      <c r="U166" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U166" t="inlineStr">
+      <c r="V166" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -19341,12 +19591,13 @@
           <t>-74.1098</t>
         </is>
       </c>
-      <c r="T167" t="inlineStr">
+      <c r="T167" t="inlineStr"/>
+      <c r="U167" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U167" t="inlineStr">
+      <c r="V167" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -19448,12 +19699,13 @@
           <t>-67.5047</t>
         </is>
       </c>
-      <c r="T168" t="inlineStr">
+      <c r="T168" t="inlineStr"/>
+      <c r="U168" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U168" t="inlineStr">
+      <c r="V168" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -19557,6 +19809,7 @@
       </c>
       <c r="T169" t="inlineStr"/>
       <c r="U169" t="inlineStr"/>
+      <c r="V169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -19654,12 +19907,13 @@
           <t>-67.3355</t>
         </is>
       </c>
-      <c r="T170" t="inlineStr">
+      <c r="T170" t="inlineStr"/>
+      <c r="U170" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U170" t="inlineStr">
+      <c r="V170" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -19761,12 +20015,13 @@
           <t>-69.0819</t>
         </is>
       </c>
-      <c r="T171" t="inlineStr">
+      <c r="T171" t="inlineStr"/>
+      <c r="U171" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U171" t="inlineStr">
+      <c r="V171" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -19868,12 +20123,13 @@
           <t>-74.452</t>
         </is>
       </c>
-      <c r="T172" t="inlineStr">
+      <c r="T172" t="inlineStr"/>
+      <c r="U172" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U172" t="inlineStr">
+      <c r="V172" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -19977,6 +20233,7 @@
       </c>
       <c r="T173" t="inlineStr"/>
       <c r="U173" t="inlineStr"/>
+      <c r="V173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -20074,12 +20331,13 @@
           <t>-59.6666</t>
         </is>
       </c>
-      <c r="T174" t="inlineStr">
+      <c r="T174" t="inlineStr"/>
+      <c r="U174" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U174" t="inlineStr">
+      <c r="V174" t="inlineStr">
         <is>
           <t>Q1_FS.xls</t>
         </is>
@@ -20181,12 +20439,13 @@
           <t>-43.4446</t>
         </is>
       </c>
-      <c r="T175" t="inlineStr">
+      <c r="T175" t="inlineStr"/>
+      <c r="U175" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U175" t="inlineStr">
+      <c r="V175" t="inlineStr">
         <is>
           <t>Q2_FS.xls</t>
         </is>
@@ -20288,12 +20547,13 @@
           <t>-33.0617</t>
         </is>
       </c>
-      <c r="T176" t="inlineStr">
+      <c r="T176" t="inlineStr"/>
+      <c r="U176" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U176" t="inlineStr">
+      <c r="V176" t="inlineStr">
         <is>
           <t>Q3_FS.xls</t>
         </is>
@@ -20397,6 +20657,7 @@
       </c>
       <c r="T177" t="inlineStr"/>
       <c r="U177" t="inlineStr"/>
+      <c r="V177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -20494,12 +20755,13 @@
           <t>-22.7338</t>
         </is>
       </c>
-      <c r="T178" t="inlineStr">
+      <c r="T178" t="inlineStr"/>
+      <c r="U178" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U178" t="inlineStr">
+      <c r="V178" t="inlineStr">
         <is>
           <t>Q1_FS.xls</t>
         </is>
@@ -20601,12 +20863,13 @@
           <t>-21.3259</t>
         </is>
       </c>
-      <c r="T179" t="inlineStr">
+      <c r="T179" t="inlineStr"/>
+      <c r="U179" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U179" t="inlineStr">
+      <c r="V179" t="inlineStr">
         <is>
           <t>Q2_FS.xls</t>
         </is>
@@ -20708,12 +20971,13 @@
           <t>-22.7589</t>
         </is>
       </c>
-      <c r="T180" t="inlineStr">
+      <c r="T180" t="inlineStr"/>
+      <c r="U180" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U180" t="inlineStr">
+      <c r="V180" t="inlineStr">
         <is>
           <t>Q3_FS.xls</t>
         </is>
@@ -20817,6 +21081,7 @@
       </c>
       <c r="T181" t="inlineStr"/>
       <c r="U181" t="inlineStr"/>
+      <c r="V181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -20914,12 +21179,13 @@
           <t>-153.4896</t>
         </is>
       </c>
-      <c r="T182" t="inlineStr">
+      <c r="T182" t="inlineStr"/>
+      <c r="U182" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U182" t="inlineStr">
+      <c r="V182" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -21021,12 +21287,13 @@
           <t>-153.2134</t>
         </is>
       </c>
-      <c r="T183" t="inlineStr">
+      <c r="T183" t="inlineStr"/>
+      <c r="U183" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U183" t="inlineStr">
+      <c r="V183" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -21128,12 +21395,13 @@
           <t>-145.746</t>
         </is>
       </c>
-      <c r="T184" t="inlineStr">
+      <c r="T184" t="inlineStr"/>
+      <c r="U184" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U184" t="inlineStr">
+      <c r="V184" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -21237,6 +21505,7 @@
       </c>
       <c r="T185" t="inlineStr"/>
       <c r="U185" t="inlineStr"/>
+      <c r="V185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -21334,12 +21603,13 @@
           <t>-95.8769</t>
         </is>
       </c>
-      <c r="T186" t="inlineStr">
+      <c r="T186" t="inlineStr"/>
+      <c r="U186" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U186" t="inlineStr">
+      <c r="V186" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -21441,12 +21711,13 @@
           <t>-77.4703</t>
         </is>
       </c>
-      <c r="T187" t="inlineStr">
+      <c r="T187" t="inlineStr"/>
+      <c r="U187" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U187" t="inlineStr">
+      <c r="V187" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -21548,12 +21819,13 @@
           <t>-69.6165</t>
         </is>
       </c>
-      <c r="T188" t="inlineStr">
+      <c r="T188" t="inlineStr"/>
+      <c r="U188" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U188" t="inlineStr">
+      <c r="V188" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -21657,6 +21929,7 @@
       </c>
       <c r="T189" t="inlineStr"/>
       <c r="U189" t="inlineStr"/>
+      <c r="V189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -21754,12 +22027,13 @@
           <t>-74.0958</t>
         </is>
       </c>
-      <c r="T190" t="inlineStr">
+      <c r="T190" t="inlineStr"/>
+      <c r="U190" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U190" t="inlineStr">
+      <c r="V190" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -21861,12 +22135,13 @@
           <t>-74.623</t>
         </is>
       </c>
-      <c r="T191" t="inlineStr">
+      <c r="T191" t="inlineStr"/>
+      <c r="U191" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U191" t="inlineStr">
+      <c r="V191" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -21968,12 +22243,13 @@
           <t>-84.7506</t>
         </is>
       </c>
-      <c r="T192" t="inlineStr">
+      <c r="T192" t="inlineStr"/>
+      <c r="U192" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U192" t="inlineStr">
+      <c r="V192" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -22077,6 +22353,7 @@
       </c>
       <c r="T193" t="inlineStr"/>
       <c r="U193" t="inlineStr"/>
+      <c r="V193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -22174,12 +22451,13 @@
           <t>-119.0582</t>
         </is>
       </c>
-      <c r="T194" t="inlineStr">
+      <c r="T194" t="inlineStr"/>
+      <c r="U194" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U194" t="inlineStr">
+      <c r="V194" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -22281,12 +22559,13 @@
           <t>-141.9209</t>
         </is>
       </c>
-      <c r="T195" t="inlineStr">
+      <c r="T195" t="inlineStr"/>
+      <c r="U195" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U195" t="inlineStr">
+      <c r="V195" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -22388,12 +22667,13 @@
           <t>-150.6563</t>
         </is>
       </c>
-      <c r="T196" t="inlineStr">
+      <c r="T196" t="inlineStr"/>
+      <c r="U196" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U196" t="inlineStr">
+      <c r="V196" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -22497,6 +22777,7 @@
       </c>
       <c r="T197" t="inlineStr"/>
       <c r="U197" t="inlineStr"/>
+      <c r="V197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -22594,12 +22875,13 @@
           <t>-147.4381</t>
         </is>
       </c>
-      <c r="T198" t="inlineStr">
+      <c r="T198" t="inlineStr"/>
+      <c r="U198" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U198" t="inlineStr">
+      <c r="V198" t="inlineStr">
         <is>
           <t>Q1_FS.xlsx</t>
         </is>
@@ -22701,12 +22983,13 @@
           <t>-124.1032</t>
         </is>
       </c>
-      <c r="T199" t="inlineStr">
+      <c r="T199" t="inlineStr"/>
+      <c r="U199" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U199" t="inlineStr">
+      <c r="V199" t="inlineStr">
         <is>
           <t>Q2_FS.xlsx</t>
         </is>
@@ -22808,12 +23091,13 @@
           <t>-94.0839</t>
         </is>
       </c>
-      <c r="T200" t="inlineStr">
+      <c r="T200" t="inlineStr"/>
+      <c r="U200" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="U200" t="inlineStr">
+      <c r="V200" t="inlineStr">
         <is>
           <t>Q3_FS.xlsx</t>
         </is>
@@ -22917,6 +23201,7 @@
       </c>
       <c r="T201" t="inlineStr"/>
       <c r="U201" t="inlineStr"/>
+      <c r="V201" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>